<commit_message>
Kit de reprise regenere : poste et statut dans le modele des agents
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/KIT-REPRISE/01-agents.xlsx
+++ b/KIT-REPRISE/01-agents.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:I1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -421,19 +421,25 @@
         <v>Date d'entrée</v>
       </c>
       <c r="G1" t="str">
+        <v>Poste</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Statut</v>
+      </c>
+      <c r="I1" t="str">
         <v>Actif</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:I4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -455,6 +461,12 @@
         <v>Date d'entrée</v>
       </c>
       <c r="G1" t="str">
+        <v>Poste</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Statut</v>
+      </c>
+      <c r="I1" t="str">
         <v>Actif</v>
       </c>
     </row>
@@ -478,6 +490,12 @@
         <v>2012-01-09</v>
       </c>
       <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v/>
+      </c>
+      <c r="I2" t="str">
         <v>Oui</v>
       </c>
     </row>
@@ -501,6 +519,12 @@
         <v>2019-09-02</v>
       </c>
       <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
         <v>Oui</v>
       </c>
     </row>
@@ -524,19 +548,25 @@
         <v>2021-04-12</v>
       </c>
       <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
         <v>Non</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <cols>
     <col min="1" max="1" width="28.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -666,24 +696,58 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Actif</v>
+        <v>Poste</v>
       </c>
       <c r="B8" t="str">
         <v>non</v>
       </c>
       <c r="C8" t="str">
+        <v>Texte</v>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Statut</v>
+      </c>
+      <c r="B9" t="str">
+        <v>non</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Texte</v>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Actif</v>
+      </c>
+      <c r="B10" t="str">
+        <v>non</v>
+      </c>
+      <c r="C10" t="str">
         <v>Oui / Non</v>
       </c>
-      <c r="D8" t="str">
-        <v/>
-      </c>
-      <c r="E8" t="str">
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>